<commit_message>
results for non-greedy version
</commit_message>
<xml_diff>
--- a/outputs/Results.xlsx
+++ b/outputs/Results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cjgry\Desktop\School Stuff\Int\int-programming\outputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644DA4AD-2249-43BF-B499-03CFC22335DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{338CE528-0E14-4B38-8329-84C29BB5553C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{FB7157C0-2B0B-40F6-8E4A-2AF8E2052130}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Size</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Initial Distance</t>
   </si>
   <si>
-    <t>Best Distance</t>
-  </si>
-  <si>
     <t>CPLEX Comparison</t>
   </si>
   <si>
@@ -99,6 +96,24 @@
   </si>
   <si>
     <t>didn't save oops</t>
+  </si>
+  <si>
+    <t>Best Distance (GREEDY)</t>
+  </si>
+  <si>
+    <t>Best Distance (normal)</t>
+  </si>
+  <si>
+    <t>N/A could not find any integer solution in about an hour</t>
+  </si>
+  <si>
+    <t>1000 took about 3 minutes for greedy</t>
+  </si>
+  <si>
+    <t>started at 12:57, ended 1:46</t>
+  </si>
+  <si>
+    <t>Ran for about an hour</t>
   </si>
 </sst>
 </file>
@@ -470,18 +485,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{693D2F79-EBFA-4FA2-A42B-1AC6BFB42BE2}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="4.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.6328125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="60.90625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="57.453125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="43.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="60.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -489,28 +505,31 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>18</v>
-      </c>
       <c r="G1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="H1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>10</v>
       </c>
@@ -521,19 +540,22 @@
         <v>12.516978039789601</v>
       </c>
       <c r="D2">
+        <v>12.516978039789601</v>
+      </c>
+      <c r="E2">
         <v>12.516999999999999</v>
       </c>
-      <c r="E2">
+      <c r="F2">
         <v>0</v>
       </c>
-      <c r="F2" t="s">
-        <v>5</v>
-      </c>
       <c r="G2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+      <c r="H2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>30</v>
       </c>
@@ -541,22 +563,25 @@
         <v>66.793163757099407</v>
       </c>
       <c r="C3">
+        <v>59.305538008862797</v>
+      </c>
+      <c r="D3">
         <v>59.810275953865201</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>59.305900000000001</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>34.729999999999997</v>
       </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
       <c r="G3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+        <v>18</v>
+      </c>
+      <c r="H3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>100</v>
       </c>
@@ -564,22 +589,25 @@
         <v>9.6911845932347003</v>
       </c>
       <c r="C4">
+        <v>9.6911845932347003</v>
+      </c>
+      <c r="D4">
         <v>8.1534128802688404</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>7.6449999999999996</v>
       </c>
-      <c r="E4">
+      <c r="F4">
         <v>0</v>
       </c>
-      <c r="F4" t="s">
-        <v>8</v>
-      </c>
       <c r="G4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+      <c r="H4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1000</v>
       </c>
@@ -587,28 +615,43 @@
         <v>29.480504892946499</v>
       </c>
       <c r="C5">
+        <v>29.480504892946499</v>
+      </c>
+      <c r="D5">
         <v>28.876640951610401</v>
       </c>
-      <c r="F5" t="s">
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="C6" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="G7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="F7" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" t="s">
         <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="F8" t="s">
-        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>